<commit_message>
Script v0.5: 6 ECTS, dates confirmed, two supervisors per group, 8 students, HPL F floor
Shorter what-you-need list; competence framework table and LLM error log
removed; no animal use anywhere, extensions start from surplus primary
material; human dataset for arm 2 is GSE228030 via the lab's HuMac pipeline.
Workbook: supervisors plural, planning wording and policy text updated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -917,7 +917,7 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Each group fills its own row with its supervisor on the planning day (Thu 18 March, afternoon) and submits the plan on Friday. The plan is the group's first deliverable. The supervisor travels with the group for the whole course and may fold in experiments the lab needs anyway; those go into the group notebook like any other experiment.</t>
+          <t>Plenary sessions (fixed layer) are mandatory. Wet-lab times listed for a group are guaranteed: hoods and cytometer slots are reserved. Everything else is orientation; if space permits, a group may shift work with its supervisors' agreement. Nobody submits a timetable.</t>
         </is>
       </c>
     </row>
@@ -1286,7 +1286,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fixed layer is drawn by staff and locked. Groups fill their own row with their supervisor on the planning day. Colours: see Legend.</t>
+          <t>Bold fixed-layer sessions are plenary and mandatory; wet-lab times listed for a group are guaranteed; everything else is orientation and may shift with the supervisors' agreement.</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1499,7 @@
       <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Group A
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B7" s="27" t="inlineStr">
@@ -1521,7 +1521,7 @@
       </c>
       <c r="G7" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisor: fill this Gantt (your row), choose the PRR axis and the extensions</t>
+          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H7" s="32" t="n"/>
@@ -1555,7 +1555,7 @@
       <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Group B
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B8" s="27" t="inlineStr">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="G8" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisor: fill this Gantt (your row), choose the PRR axis and the extensions</t>
+          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H8" s="32" t="n"/>
@@ -1611,7 +1611,7 @@
       <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Group C
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B9" s="27" t="inlineStr">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="G9" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisor: fill this Gantt (your row), choose the PRR axis and the extensions</t>
+          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H9" s="32" t="n"/>
@@ -1667,7 +1667,7 @@
       <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Group D
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B10" s="27" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="G10" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisor: fill this Gantt (your row), choose the PRR axis and the extensions</t>
+          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H10" s="32" t="n"/>
@@ -1901,7 +1901,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fixed layer is drawn by staff and locked. Groups fill their own row with their supervisor on the planning day. Colours: see Legend.</t>
+          <t>Bold fixed-layer sessions are plenary and mandatory; wet-lab times listed for a group are guaranteed; everything else is orientation and may shift with the supervisors' agreement.</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2278,7 @@
       <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Group A
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B7" s="36" t="inlineStr">
@@ -2382,7 +2382,7 @@
       <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Group B
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B8" s="36" t="inlineStr">
@@ -2486,7 +2486,7 @@
       <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Group C
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B9" s="31" t="inlineStr">
@@ -2590,7 +2590,7 @@
       <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Group D
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B10" s="31" t="inlineStr">
@@ -2969,7 +2969,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fixed layer is drawn by staff and locked. Groups fill their own row with their supervisor on the planning day. Colours: see Legend.</t>
+          <t>Bold fixed-layer sessions are plenary and mandatory; wet-lab times listed for a group are guaranteed; everything else is orientation and may shift with the supervisors' agreement.</t>
         </is>
       </c>
     </row>
@@ -3434,7 +3434,7 @@
       <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Group A
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B7" s="31" t="inlineStr">
@@ -3558,7 +3558,7 @@
       <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Group B
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B8" s="31" t="inlineStr">
@@ -3682,7 +3682,7 @@
       <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Group C
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B9" s="37" t="inlineStr">
@@ -3802,7 +3802,7 @@
       <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Group D
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B10" s="37" t="inlineStr">
@@ -4108,9 +4108,9 @@
   </sheetData>
   <mergeCells count="70">
     <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="AH3:AO3"/>
     <mergeCell ref="AH10:AJ10"/>
     <mergeCell ref="AH12:AO12"/>
     <mergeCell ref="R11:Y11"/>
@@ -4244,7 +4244,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fixed layer is drawn by staff and locked. Groups fill their own row with their supervisor on the planning day. Colours: see Legend.</t>
+          <t>Bold fixed-layer sessions are plenary and mandatory; wet-lab times listed for a group are guaranteed; everything else is orientation and may shift with the supervisors' agreement.</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       <c r="A7" s="26" t="inlineStr">
         <is>
           <t>Group A
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B7" s="38" t="inlineStr">
@@ -4845,7 +4845,7 @@
       <c r="A8" s="26" t="inlineStr">
         <is>
           <t>Group B
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B8" s="38" t="inlineStr">
@@ -4977,7 +4977,7 @@
       <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Group C
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B9" s="31" t="inlineStr">
@@ -5109,7 +5109,7 @@
       <c r="A10" s="26" t="inlineStr">
         <is>
           <t>Group D
-supervisor: ________</t>
+supervisors: ______ / ______</t>
         </is>
       </c>
       <c r="B10" s="31" t="inlineStr">
@@ -5416,9 +5416,9 @@
   <mergeCells count="67">
     <mergeCell ref="V10:X10"/>
     <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="AH3:AO3"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="R11:Y11"/>
     <mergeCell ref="V9:X9"/>

</xml_diff>

<commit_message>
Schedule: group formation at 14:00 on day 1, names on lectures and seminars, tbd where open
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -1112,7 +1112,7 @@
       <c r="D4" s="17" t="n"/>
       <c r="E4" s="18" t="inlineStr">
         <is>
-          <t>Welcome, lectures, planning with supervisor</t>
+          <t>Welcome, lectures, group formation, planning with supervisor</t>
         </is>
       </c>
       <c r="F4" s="19" t="inlineStr">
@@ -1464,22 +1464,26 @@
       </c>
       <c r="B6" s="27" t="inlineStr">
         <is>
-          <t>Welcome, safety briefing, group formation</t>
+          <t>Welcome and safety briefing (Tea Kocijan)</t>
         </is>
       </c>
       <c r="C6" s="27" t="inlineStr">
         <is>
-          <t>Lecture: tissue macrophages and nomenclature</t>
+          <t>Lecture: tissue macrophages and nomenclature (Joel Zindel)</t>
         </is>
       </c>
       <c r="D6" s="28" t="n"/>
       <c r="E6" s="40" t="n"/>
       <c r="F6" s="27" t="inlineStr">
         <is>
-          <t>Lecture: the techniques of this course, one slide per method</t>
-        </is>
-      </c>
-      <c r="G6" s="17" t="n"/>
+          <t>Lecture: the techniques of this course, one slide per method (Agnes Huber, Brooke Slade)</t>
+        </is>
+      </c>
+      <c r="G6" s="27" t="inlineStr">
+        <is>
+          <t>Group formation</t>
+        </is>
+      </c>
       <c r="H6" s="17" t="n"/>
       <c r="I6" s="17" t="n"/>
       <c r="J6" s="17" t="n"/>
@@ -1488,7 +1492,7 @@
       <c r="M6" s="41" t="n"/>
       <c r="N6" s="29" t="inlineStr">
         <is>
-          <t>Facility lecture: flow cytometry and FlowJo [TODO: confirm slot with the facility]</t>
+          <t>Facility lecture: flow cytometry and FlowJo (Florian Mair) [TODO: confirm slot with the facility]</t>
         </is>
       </c>
       <c r="O6" s="28" t="n"/>
@@ -1521,7 +1525,7 @@
       </c>
       <c r="G7" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
+          <t>Group formation at 14:00, then experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H7" s="32" t="n"/>
@@ -1577,7 +1581,7 @@
       </c>
       <c r="G8" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
+          <t>Group formation at 14:00, then experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H8" s="32" t="n"/>
@@ -1633,7 +1637,7 @@
       </c>
       <c r="G9" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
+          <t>Group formation at 14:00, then experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H9" s="32" t="n"/>
@@ -1689,7 +1693,7 @@
       </c>
       <c r="G10" s="31" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisors: choose your PRR axis and your extensions</t>
+          <t>Group formation at 14:00, then experiment planning with your supervisors: choose your PRR axis and your extensions</t>
         </is>
       </c>
       <c r="H10" s="32" t="n"/>
@@ -1728,7 +1732,7 @@
       </c>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>Rooms, safety officer, group list. Supervisors sit with their group from 14:00.</t>
+          <t>Rooms, safety officer. Groups formed at 14:00; supervisors sit with their group from then on.</t>
         </is>
       </c>
       <c r="C11" s="32" t="n"/>
@@ -2226,7 +2230,7 @@
       <c r="D6" s="17" t="n"/>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>IMHS Lunch Seminar</t>
+          <t>IMHS Lunch Seminar (HPL D32/34)</t>
         </is>
       </c>
       <c r="F6" s="17" t="n"/>
@@ -2242,12 +2246,12 @@
       <c r="P6" s="17" t="n"/>
       <c r="Q6" s="27" t="inlineStr">
         <is>
-          <t>Cutting Edge Immunology Seminar 16:30-17:30</t>
+          <t>Cutting Edge Immunology Seminar 16:30-17:30 (tbd)</t>
         </is>
       </c>
       <c r="R6" s="27" t="inlineStr">
         <is>
-          <t>Lecture: tissue repair I, macrophages in injury and repair</t>
+          <t>Lecture: tissue repair I, macrophages in injury and repair (tbd)</t>
         </is>
       </c>
       <c r="S6" s="17" t="n"/>
@@ -2259,7 +2263,7 @@
       <c r="Y6" s="17" t="n"/>
       <c r="Z6" s="27" t="inlineStr">
         <is>
-          <t>Journal club 1: the M1/M2 nomenclature revision [TODO: paper]; one group presents, all read</t>
+          <t>Journal club 1 (tbd): the M1/M2 nomenclature revision [TODO: paper]; one group presents, all read</t>
         </is>
       </c>
       <c r="AA6" s="17" t="n"/>
@@ -3366,7 +3370,7 @@
       <c r="D6" s="17" t="n"/>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>IMHS Lunch Seminar</t>
+          <t>IMHS Lunch Seminar (HPL D32/34)</t>
         </is>
       </c>
       <c r="F6" s="17" t="n"/>
@@ -3375,7 +3379,7 @@
       <c r="I6" s="17" t="n"/>
       <c r="J6" s="27" t="inlineStr">
         <is>
-          <t>Lecture: single-cell transcriptomics for immunologists, what a signature score means</t>
+          <t>Lecture: single-cell transcriptomics for immunologists, what a signature score means (tbd)</t>
         </is>
       </c>
       <c r="K6" s="17" t="n"/>
@@ -3386,7 +3390,7 @@
       <c r="P6" s="17" t="n"/>
       <c r="Q6" s="27" t="inlineStr">
         <is>
-          <t>Cutting Edge Immunology Seminar 16:30-17:30</t>
+          <t>Cutting Edge Immunology Seminar 16:30-17:30 (tbd)</t>
         </is>
       </c>
       <c r="R6" s="17" t="n"/>
@@ -3407,7 +3411,7 @@
       <c r="Y6" s="28" t="n"/>
       <c r="Z6" s="27" t="inlineStr">
         <is>
-          <t>Journal club 2: the peritoneal injury single-cell paper behind GSE186658 [TODO: paper]; one group presents, all read</t>
+          <t>Journal club 2 (tbd): the peritoneal injury single-cell paper behind GSE186658 [TODO: paper]; one group presents, all read</t>
         </is>
       </c>
       <c r="AA6" s="17" t="n"/>
@@ -4108,9 +4112,9 @@
   </sheetData>
   <mergeCells count="70">
     <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="B13:AO13"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="AH3:AO3"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="B13:AO13"/>
     <mergeCell ref="AH10:AJ10"/>
     <mergeCell ref="AH12:AO12"/>
     <mergeCell ref="R11:Y11"/>
@@ -4641,7 +4645,7 @@
       <c r="D6" s="17" t="n"/>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>IMHS Lunch Seminar</t>
+          <t>IMHS Lunch Seminar (HPL D32/34)</t>
         </is>
       </c>
       <c r="F6" s="17" t="n"/>
@@ -4657,12 +4661,12 @@
       <c r="P6" s="17" t="n"/>
       <c r="Q6" s="27" t="inlineStr">
         <is>
-          <t>Cutting Edge Immunology Seminar 16:30-17:30</t>
+          <t>Cutting Edge Immunology Seminar 16:30-17:30 (tbd)</t>
         </is>
       </c>
       <c r="R6" s="27" t="inlineStr">
         <is>
-          <t>Lecture: scientific writing, from data to argument, poster structure, figure design, honest limits</t>
+          <t>Lecture: scientific writing, from data to argument, poster structure, figure design, honest limits (tbd)</t>
         </is>
       </c>
       <c r="S6" s="41" t="n"/>
@@ -4683,7 +4687,7 @@
       <c r="AD6" s="41" t="n"/>
       <c r="AE6" s="27" t="inlineStr">
         <is>
-          <t>Recap and Q&amp;A: the course in one hour, then open questions with the teaching staff</t>
+          <t>Recap and Q&amp;A (tbd): the course in one hour, then open questions with the teaching staff</t>
         </is>
       </c>
       <c r="AF6" s="30" t="n"/>
@@ -5416,9 +5420,9 @@
   <mergeCells count="67">
     <mergeCell ref="V10:X10"/>
     <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="B13:AO13"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="AH3:AO3"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="B13:AO13"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="R11:Y11"/>
     <mergeCell ref="V9:X9"/>

</xml_diff>

<commit_message>
Written exam Friday 13:00, poster printing by the groups via Signprint
- Fri 16 April: written exam at 13:00 (individual), poster session and prize
  from 14:00, apéro at 16:00.
- No printing deadline on the plan: each group commits the PDF to its branch
  and orders the print at signprint.ch when ready; poster guide updated.
- README Section 7: written exam 50%, group grade from the branch (poster and
  the way there) 50%. Poster printing dropped from the open items.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,6 +507,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1156,7 +1162,7 @@
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>[TODO] Poster printing: printer. Deadline is Thu 15 Apr 14:00 (poster PDF committed to the group branch).</t>
+          <t>Poster printing: each group orders its own poster (signprint.ch, see poster/README.md) in time for the poster session on Fri 16 April 14:00; the PDF is committed to the group branch first. No deadline on the plan.</t>
         </is>
       </c>
     </row>
@@ -1340,12 +1346,12 @@
       </c>
       <c r="E8" s="51" t="inlineStr">
         <is>
-          <t>Poster production; printing deadline 14:00; recap and Q&amp;A</t>
+          <t>Poster production; print when ready; recap and Q&amp;A</t>
         </is>
       </c>
       <c r="F8" s="46" t="inlineStr">
         <is>
-          <t>Clean-up, feedback; poster presentations, prize, Apéro</t>
+          <t>Clean-up, feedback; written exam 13:00; poster session, prize, Apéro</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1389,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>Week 1: orientation (Thu 18 - Fri 19 March 2027)</t>
         </is>
@@ -1584,7 +1590,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>Week 2: Exp 1, establish the line (Tue 23 - Thu 25 March 2027)</t>
         </is>
@@ -1840,7 +1846,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>Week 3: Exp 2, challenge and read out (Tue 6 - Fri 9 April 2027)</t>
         </is>
@@ -2132,7 +2138,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>Week 4: extensions, poster, presentations (Tue 13 - Fri 16 April 2027)</t>
         </is>
@@ -2282,12 +2288,12 @@
       </c>
       <c r="D8" s="51" t="inlineStr">
         <is>
-          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch</t>
+          <t>Poster production, continued. Print when you are ready (poster guide); the PDF goes to the group branch first</t>
         </is>
       </c>
       <c r="E8" s="46" t="inlineStr">
         <is>
-          <t>Poster presentations and discussion; prize</t>
+          <t>Written exam, individual [TODO: duration and room]</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2310,11 @@
           <t>Recap and Q&amp;A (tbd): the course in one hour, then open questions with the teaching staff</t>
         </is>
       </c>
-      <c r="E9" s="65" t="n"/>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>Poster session: presentations and discussion; prize</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="64" customHeight="1">
       <c r="A10" s="45" t="inlineStr">
@@ -2357,17 +2367,17 @@
       </c>
       <c r="C12" s="55" t="inlineStr">
         <is>
-          <t>Poster template distributed, printing booked [TODO: printer]. Rescue groups: cytometer slot [TODO: facility], ELISA Wed, result on the poster by Thursday.</t>
+          <t>Poster template distributed. Rescue groups: cytometer slot [TODO: facility], ELISA Wed, result on the poster by Thursday.</t>
         </is>
       </c>
       <c r="D12" s="55" t="inlineStr">
         <is>
-          <t>Posters printed Thu after 14:00 [TODO: printer].</t>
+          <t>Printing is each group's own business (signprint.ch, see the poster guide). Poster boards ready.</t>
         </is>
       </c>
       <c r="E12" s="55" t="inlineStr">
         <is>
-          <t>Jury, prize, evaluation form, clean-up checklist. Apéro ordered [TODO: catering].</t>
+          <t>Exam papers, jury, prize, evaluation form, clean-up checklist. Apéro ordered [TODO: catering].</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2399,7 @@
       </c>
       <c r="D13" s="55" t="inlineStr">
         <is>
-          <t>Conference room HPL F22 for lectures and dry lab. Printer [TODO]. Poster boards.</t>
+          <t>Conference room HPL F22 for lectures and dry lab. Poster boards.</t>
         </is>
       </c>
       <c r="E13" s="55" t="inlineStr">
@@ -2401,10 +2411,10 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="D4:D6"/>
+    <mergeCell ref="E9:E10"/>
     <mergeCell ref="D10:D11"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="B4:B6"/>
-    <mergeCell ref="E8:E10"/>
     <mergeCell ref="E4:E5"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="B8:B10"/>

</xml_diff>

<commit_message>
WIP: plan v2 schedule and stock-flask protocols
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,6 +507,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -937,7 +943,7 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Wet lab Exp 1: establish the line (growth curve, freeze, re-thaw)</t>
+          <t>Wet lab Exp 1: polarize and characterize (plate with the polarizer, harvest, stain, acquire)</t>
         </is>
       </c>
     </row>
@@ -949,7 +955,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Wet lab Exp 2: challenge, read out (flow cytometry, ELISA)</t>
+          <t>Wet lab Exp 2: polarize and challenge (plate, stimulate, harvest, ELISA)</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1015,7 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>One sheet per week: one column per day, one row per hour. Course hours Tue 13:00-17:00 and Wed-Fri 09:00-17:00; Monday and Tuesday morning are the students' other lectures. Below the hour grid: a staff row and a resources row, one cell per day.</t>
+          <t>One sheet per week: one column per day, one row per hour, 08:00 to 17:00 (Tuesdays from 13:00; Monday and Tuesday morning are the students' other lectures). Every full day opens with a self-study hour. Below the hour grid: a staff row and a resources row, one cell per day.</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1027,7 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Lecture slots, journal clubs, facility lecture, cytometer slots, the Tuesday Cutting Edge Immunology Seminar (16:30-17:30) in weeks 3 and 4, writing lecture, recap, presentations. Drawn by the teaching staff, dark cells, thick border, locked. Everything else is flexible.</t>
+          <t>Lecture slots, the facility lecture, cytometer slots and the FlowJo session, journal club, the Tuesday Cutting Edge Immunology Seminar (16:30-17:30) in weeks 3 and 4, the publish-or-perish discussion, exam, poster session. Drawn by the teaching staff, dark cells, thick border, locked. Everything else is flexible.</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1063,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Exp 1 (week 2): establish the RAW 264.7 line. Thaw on Tuesday afternoon, five trypan-blue counts to Thursday afternoon (growth curve, doubling time), MTT columns as a second readout, freeze your own vials on Thursday; viability of your vial after the break is the third readout. Exp 2 (week 3): plate RAW cells, spin, 2 h adhesion, overnight LPS challenge; readouts flow cytometry and ELISA. Polarization (P04) and Griess (P07) are extensions. Protocol IDs (P01...) refer to protocols/ in the course repository.</t>
+          <t>Exp 1 (week 2): polarize and characterize. Plate from the group's stock with the polarizer in the seeding suspension, vehicle and LPS controls beside it; harvest, stain, acquire; FlowJo; decide to stick or pivot before the break. Exp 2 (week 3): polarize and challenge. Plate with the polarizer on Tuesday, challenge on Wednesday with the group's stimulus and optional inhibitor (LPS on M(-) shared by all), overnight with an IL-6 readout by default or 6 h with TNF; ELISA on Thursday. Week 4: repeat, add, or wrap up. Menus in P04 and P05. Protocol IDs (P01...) refer to protocols/ in the course repository.</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1075,7 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Week 1: environment and templates. Week 2: scRNA-seq part 1 (QC), FlowJo on example data, growth curve. Week 3: scRNA-seq part 2 (signatures from the bulk RAW 264.7 dataset) during the ELISA incubations, own flow and ELISA data on Friday. Week 4: scRNA-seq part 3 (scoring of the tissue macrophages), extension analysis and poster figures. Downtime at any point: poster introduction and significance.</t>
+          <t>Week 1: environment and templates. Week 2: scRNA-seq part 1 (QC) in the afternoon dry-lab slots, FlowJo on the own data. Week 3: scRNA-seq part 2 (signatures from the bulk RAW 264.7 dataset) during the challenge and the ELISA incubations, own ELISA data on Friday. Week 4: scRNA-seq part 3 (scoring of the tissue macrophages), wrap up of code, figures and poster.</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1087,7 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>A group whose Exp 2 failed repeats it in week 4: plate, spin and challenge Tue 13 April at 13:00, harvest and stain Wed 14 at 09:00, ELISA Wed 14, acquisition in a week-4 cytometer slot [TODO: facility].</t>
+          <t>A group whose polarization or challenge failed repeats it in week 4, Tuesday 13:00 to Wednesday, as agreed with the supervisor on Friday 9 April; never at the cost of wrapping up.</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1099,7 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Fri 26 March to Sun 4 April. No course, no cultures. Staff thaw backup RAW on Wed 31 March and split Fri 2 April [TODO: confirm dates with the department].</t>
+          <t>Fri 26 March to Sun 4 April. No course. The staff carry the groups' stock flasks over the break (split every 2 to 3 days, backup vials frozen on Thu 25 March).</t>
         </is>
       </c>
     </row>
@@ -1107,14 +1113,14 @@
     <row r="24">
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>[TODO] Cytometer slots: dates and times from the facility (week 3 Thursday 8 April, 10:00-12:00 and 13:00-15:00; rescue and extension slots week 4).</t>
+          <t>[TODO] Cytometer: two slots of 1.5 h on Thu 25 March 09:00-12:00 (two groups each); FlowJo teaching seats for the session on Thu 25 March 13:00 (Florian Mair). Week 3 and 4 slots only through the regular booking calendar.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>[TODO] Facility lecture: slot on Wed 24 March 13:00.</t>
+          <t>[TODO] Facility lecture: slot on Wed 24 March 09:00.</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1234,12 @@
       <c r="D4" s="41" t="n"/>
       <c r="E4" s="46" t="inlineStr">
         <is>
-          <t>Welcome, lectures, group formation, planning with supervisor</t>
+          <t>Welcome, lecture, group formation; the pathway drawing and the menu choices</t>
         </is>
       </c>
       <c r="F4" s="47" t="inlineStr">
         <is>
-          <t>Hands-on cell-culture introduction on the staff culture; dry lab setup; plans submitted</t>
+          <t>Hands-on cell culture; thaw and seed the group's stock flask; dry lab setup; plan committed</t>
         </is>
       </c>
     </row>
@@ -1250,17 +1256,17 @@
       </c>
       <c r="C5" s="47" t="inlineStr">
         <is>
-          <t>Morning: other lectures. 13:00 Exp 1: thaw, T0, seed</t>
+          <t>Morning: other lectures. 13:00 plate with the polarizer; dry lab</t>
         </is>
       </c>
       <c r="D5" s="47" t="inlineStr">
         <is>
-          <t>Exp 1: counts 1 and 2, MTT, medium change; flow lecture</t>
-        </is>
-      </c>
-      <c r="E5" s="47" t="inlineStr">
-        <is>
-          <t>Exp 1: counts 3 and 4, freeze; debrief</t>
+          <t>Facility lecture; harvest, stain, fix</t>
+        </is>
+      </c>
+      <c r="E5" s="56" t="inlineStr">
+        <is>
+          <t>Flow acquisition; FlowJo session; journal club and debrief: stick or pivot</t>
         </is>
       </c>
       <c r="F5" s="48" t="inlineStr">
@@ -1277,7 +1283,7 @@
       </c>
       <c r="B6" s="48" t="inlineStr">
         <is>
-          <t>Break 26 Mar - 4 Apr; staff thaw backup cells</t>
+          <t>Break 26 Mar - 4 Apr; staff carry the stock flasks</t>
         </is>
       </c>
       <c r="C6" s="41" t="n"/>
@@ -1298,22 +1304,22 @@
       </c>
       <c r="C7" s="49" t="inlineStr">
         <is>
-          <t>Morning: other lectures. 13:00 plate, spin, 2 h, LPS challenge overnight; re-thaw own vial</t>
+          <t>Morning: other lectures. 13:00 plate with the chosen polarizer; passage the stock</t>
         </is>
       </c>
       <c r="D7" s="49" t="inlineStr">
         <is>
-          <t>Harvest cells and supernatants; flow staining and fix; ELISA plates coated</t>
+          <t>Challenge (overnight IL-6 default, 6 h TNF alternative); lecture; coat ELISA plates</t>
         </is>
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>Flow acquisition (A+B morning, C+D afternoon); ELISA in the other half</t>
+          <t>Harvest; ELISA with dry lab in the incubations</t>
         </is>
       </c>
       <c r="F7" s="49" t="inlineStr">
         <is>
-          <t>FlowJo session; ELISA analysis; debrief</t>
+          <t>ELISA analysis; poster: what is missing; debrief</t>
         </is>
       </c>
     </row>
@@ -1330,36 +1336,36 @@
       </c>
       <c r="C8" s="50" t="inlineStr">
         <is>
-          <t>Morning: other lectures. 13:00 extensions or rescue path</t>
+          <t>Morning: other lectures. 13:00 optional repeat, third experiment, or dry lab</t>
         </is>
       </c>
       <c r="D8" s="51" t="inlineStr">
         <is>
-          <t>Writing lecture; extensions; poster; failure round</t>
+          <t>Optional harvest and ELISA; wrap up; publish or perish</t>
         </is>
       </c>
       <c r="E8" s="51" t="inlineStr">
         <is>
-          <t>Poster production; printing deadline 14:00; recap and Q&amp;A</t>
+          <t>Wrap up: code, figures, poster; print when ready</t>
         </is>
       </c>
       <c r="F8" s="46" t="inlineStr">
         <is>
-          <t>Clean-up, feedback; poster presentations, prize, Apéro</t>
+          <t>Lab cleaning; finish the branch; written exam 13:00; poster session; 360° feedback; Apéro</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Course weeks run Tuesday 13:00 to Friday 17:00; Monday and Tuesday morning are the students' other lectures. All four groups follow the same plan, each at its own hood; see the week sheets.</t>
+          <t>Course days run 08:00 to 17:00, Tuesdays from 13:00; Monday and Tuesday morning are the students' other lectures. Every full day opens with a self-study hour. All four groups follow the same plan, each at its own hood; see the week sheets.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Course hours Tue 13:00-17:00, Wed-Fri 09:00-17:00, lunch 12:00-13:00. Lectures and dry lab in conference room HPL F22, bench in HPL F27.2. Cutting Edge Immunology Seminar Tue 16:30-17:30 in weeks 3 and 4.</t>
+          <t>Lectures and dry lab in conference room HPL F22, bench in HPL F27.2. Cutting Edge Immunology Seminar Tue 16:30-17:30 in weeks 3 and 4.</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1383,7 +1389,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
+      <c r="A1" s="68" t="inlineStr">
         <is>
           <t>Week 1: orientation (Thu 18 - Fri 19 March 2027)</t>
         </is>
@@ -1420,136 +1426,153 @@
     <row r="4" ht="64" customHeight="1">
       <c r="A4" s="45" t="inlineStr">
         <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="46" t="inlineStr">
-        <is>
-          <t>Welcome and safety briefing (Tea Kocijan)</t>
-        </is>
-      </c>
-      <c r="C4" s="47" t="inlineStr">
-        <is>
-          <t>Hands-on introduction to mammalian cell culture with the staff culture: hood and sterile technique, microscope, P02 scrape, count, split and seed, cell counter. Lab tour.</t>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
+        </is>
+      </c>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
         </is>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="45" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B5" s="46" t="inlineStr">
         <is>
-          <t>Lecture: tissue macrophages and nomenclature (Joel Zindel)</t>
-        </is>
-      </c>
-      <c r="C5" s="65" t="n"/>
+          <t>Welcome and safety briefing (Tea Kocijan)</t>
+        </is>
+      </c>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t>Hands-on cell culture with the staff culture: hood and sterile technique, microscope, P02 scrape, count, split and seed, cell counter. Then P01: thaw and seed your group's stock flask (course passage 0). Lab tour.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="64" customHeight="1">
       <c r="A6" s="45" t="inlineStr">
         <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="B6" s="66" t="n"/>
-      <c r="C6" s="66" t="n"/>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B6" s="46" t="inlineStr">
+        <is>
+          <t>Lecture: tissue macrophages and nomenclature (Joel Zindel)</t>
+        </is>
+      </c>
+      <c r="C6" s="65" t="n"/>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="45" t="inlineStr">
         <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="B7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="C7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="n"/>
+      <c r="C7" s="66" t="n"/>
     </row>
     <row r="8" ht="64" customHeight="1">
       <c r="A8" s="45" t="inlineStr">
         <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="B8" s="46" t="inlineStr">
-        <is>
-          <t>Group formation</t>
-        </is>
-      </c>
-      <c r="C8" s="54" t="inlineStr">
-        <is>
-          <t>Dry lab setup: clone the course repository, build the environment with your chatty, run the ELISA template on example data. Group plan submitted at 17:00.</t>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
         </is>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1">
       <c r="A9" s="45" t="inlineStr">
         <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="B9" s="54" t="inlineStr">
-        <is>
-          <t>Experiment planning with your supervisors: choose your PRR axis and your extension. Read P01, P02 and P09 for Friday and Tuesday.</t>
-        </is>
-      </c>
-      <c r="C9" s="65" t="n"/>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B9" s="46" t="inlineStr">
+        <is>
+          <t>Group formation</t>
+        </is>
+      </c>
+      <c r="C9" s="54" t="inlineStr">
+        <is>
+          <t>Dry lab setup: clone the course repository, build the environment with your chatty, run the ELISA template on example data. Group plan (the drawing and your menu choices) committed to the group branch at 17:00.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="64" customHeight="1">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="B10" s="65" t="n"/>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B10" s="54" t="inlineStr">
+        <is>
+          <t>Experiment planning with your supervisors: hand-draw the pathway you will test (ligand, receptor, output, how an inhibitor proves it, where the polarizer acts), pick your polarizer, stimulus and cytokine (P04, P05, P06). Read P01, P02 and P08 for Friday and Tuesday.</t>
+        </is>
+      </c>
       <c r="C10" s="65" t="n"/>
     </row>
     <row r="11" ht="64" customHeight="1">
       <c r="A11" s="45" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B11" s="65" t="n"/>
+      <c r="C11" s="65" t="n"/>
+    </row>
+    <row r="12" ht="64" customHeight="1">
+      <c r="A12" s="45" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="B11" s="66" t="n"/>
-      <c r="C11" s="66" t="n"/>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="45" t="inlineStr">
+      <c r="B12" s="66" t="n"/>
+      <c r="C12" s="66" t="n"/>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>Staff</t>
         </is>
       </c>
-      <c r="B12" s="55" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
         <is>
           <t>Rooms, safety officer. Groups formed at 13:00; supervisors sit with their group from then on.</t>
         </is>
       </c>
-      <c r="C12" s="55" t="inlineStr">
-        <is>
-          <t>Staff culture split and counted, one flask per group at 09:00. Dry lab: walk around, unblock installs. Fallback environment ready [TODO]. Collect the group plans at 17:00.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="45" t="inlineStr">
+      <c r="C13" s="55" t="inlineStr">
+        <is>
+          <t>One low-passage vial per group. Supervisors carry the stock flasks over the weekend and the break: split every 2 to 3 days, course passage counted from this thaw. Dry lab: unblock installs; fallback environment ready [TODO]. Collect the plans at 17:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="45" t="inlineStr">
         <is>
           <t>Resources</t>
         </is>
       </c>
-      <c r="B13" s="55" t="inlineStr">
+      <c r="B14" s="55" t="inlineStr">
         <is>
           <t>Conference room HPL F22 for lectures and dry lab.</t>
         </is>
       </c>
-      <c r="C13" s="55" t="inlineStr">
+      <c r="C14" s="55" t="inlineStr">
         <is>
           <t>4 hoods HPL F27.2, one per group, available at all times. Cell counter. Conference room HPL F22 for lectures and dry lab. Own laptops, Wi-Fi.</t>
         </is>
@@ -1557,12 +1580,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="C9:C12"/>
     <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="B6:B7"/>
     <mergeCell ref="A2:C2"/>
-    <mergeCell ref="C8:C11"/>
-    <mergeCell ref="B9:B11"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C4:C6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1574,7 +1597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1584,9 +1607,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
-        <is>
-          <t>Week 2: Exp 1, establish the line (Tue 23 - Thu 25 March 2027)</t>
+      <c r="A1" s="68" t="inlineStr">
+        <is>
+          <t>Week 2: polarize and characterize (Tue 23 - Thu 25 March 2027)</t>
         </is>
       </c>
       <c r="B1" s="32" t="n"/>
@@ -1628,7 +1651,7 @@
     <row r="4" ht="64" customHeight="1">
       <c r="A4" s="45" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="B4" s="48" t="inlineStr">
@@ -1636,188 +1659,201 @@
           <t>Your other lectures (not course time)</t>
         </is>
       </c>
-      <c r="C4" s="47" t="inlineStr">
-        <is>
-          <t>P01 Count 1. P09 Seed the standard curve, MTT on column 1</t>
-        </is>
-      </c>
-      <c r="D4" s="47" t="inlineStr">
-        <is>
-          <t>P01 Count 3. P09 MTT on column 2 (read 12:30)</t>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
         </is>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="45" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B5" s="65" t="n"/>
-      <c r="C5" s="47" t="inlineStr">
-        <is>
-          <t>Inspect the flask, medium change. P09 MTT on the standard curve at 11:00; reads at 12:30 and 14:30</t>
-        </is>
-      </c>
-      <c r="D5" s="46" t="inlineStr">
-        <is>
-          <t>Journal club 1 (tbd): the M1/M2 nomenclature revision [TODO: paper]; one group presents, all read</t>
+      <c r="C5" s="56" t="inlineStr">
+        <is>
+          <t>Facility lecture: flow cytometry and FlowJo (Florian Mair) [TODO: confirm slot]</t>
+        </is>
+      </c>
+      <c r="D5" s="56" t="inlineStr">
+        <is>
+          <t>P08 Acquisition at the facility, two batches of 1.5 h, two groups each [TODO: reservation]</t>
         </is>
       </c>
     </row>
     <row r="6" ht="64" customHeight="1">
       <c r="A6" s="45" t="inlineStr">
         <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="B6" s="66" t="n"/>
-      <c r="C6" s="66" t="n"/>
-      <c r="D6" s="47" t="inlineStr">
-        <is>
-          <t>P03 Freeze your own vials from the flask. Clean-up</t>
-        </is>
-      </c>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B6" s="65" t="n"/>
+      <c r="C6" s="47" t="inlineStr">
+        <is>
+          <t>P08 Harvest the adherent cells, count, viability dye, Fc block, surface stain</t>
+        </is>
+      </c>
+      <c r="D6" s="65" t="n"/>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="45" t="inlineStr">
         <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="B7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="C7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="D7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="n"/>
+      <c r="C7" s="66" t="n"/>
+      <c r="D7" s="66" t="n"/>
     </row>
     <row r="8" ht="64" customHeight="1">
       <c r="A8" s="45" t="inlineStr">
         <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="B8" s="47" t="inlineStr">
-        <is>
-          <t>P01 Thaw your own vial, count (T0), seed the flask and the counting wells. P09 Seed the MTT growth-curve columns.</t>
-        </is>
-      </c>
-      <c r="C8" s="56" t="inlineStr">
-        <is>
-          <t>Facility lecture: flow cytometry and FlowJo (Florian Mair) [TODO: confirm slot with the facility]</t>
-        </is>
-      </c>
-      <c r="D8" s="54" t="inlineStr">
-        <is>
-          <t>Dry lab: FlowJo on example data. Growth curve and doubling time from your counts. Poster: why does this matter (significance). P09 MTT on column 3 at 12:30, read 16:00</t>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
         </is>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1">
       <c r="A9" s="45" t="inlineStr">
         <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="B9" s="65" t="n"/>
-      <c r="C9" s="54" t="inlineStr">
-        <is>
-          <t>Dry lab: scRNA-seq part 1, load the preprocessed object, QC figure. Poster: draft the introduction. P01 Count 2 at 15:00</t>
-        </is>
-      </c>
-      <c r="D9" s="66" t="n"/>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t>P02 and P04: plate cells from your stock with the polarizer already in the seeding suspension. Vehicle control, M(pol) and LPS control on the flow plate (6- or 12-well). Plate-and-polarize in one step, about 19 h. Wet-lab goal: plate at a defined density with a stimulus.</t>
+        </is>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t>P08 continued: optional Arg1 fix and perm, fix, store at 4 °C until acquisition. Wet-lab goal: harvest, staining, fixation. Staining plan and FMOs in the notebook.</t>
+        </is>
+      </c>
+      <c r="D9" s="56" t="inlineStr">
+        <is>
+          <t>FlowJo session: gating, FMOs, export statistics; the first figure [TODO: check with Florian Mair the available teaching seats]. Wet-lab goal: acquisition and gating.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="64" customHeight="1">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="B10" s="65" t="n"/>
-      <c r="C10" s="65" t="n"/>
-      <c r="D10" s="47" t="inlineStr">
-        <is>
-          <t>P01 Count 4, the last point. Discard the counting wells; nothing stays in culture over the break</t>
-        </is>
-      </c>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B10" s="66" t="n"/>
+      <c r="C10" s="66" t="n"/>
+      <c r="D10" s="65" t="n"/>
     </row>
     <row r="11" ht="64" customHeight="1">
       <c r="A11" s="45" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B11" s="54" t="inlineStr">
+        <is>
+          <t>Dry lab: scRNA-seq part 1, load the preprocessed object, QC figure. If the bench runs over, the dry lab moves home.</t>
+        </is>
+      </c>
+      <c r="C11" s="54" t="inlineStr">
+        <is>
+          <t>Dry lab: scRNA-seq part 1 continued; poster: draft the introduction. If the bench runs over, the dry lab moves home.</t>
+        </is>
+      </c>
+      <c r="D11" s="66" t="n"/>
+    </row>
+    <row r="12" ht="64" customHeight="1">
+      <c r="A12" s="45" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="B11" s="66" t="n"/>
-      <c r="C11" s="66" t="n"/>
-      <c r="D11" s="46" t="inlineStr">
-        <is>
-          <t>Debrief week 2: what worked, plan for Exp 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="45" t="inlineStr">
+      <c r="B12" s="66" t="n"/>
+      <c r="C12" s="66" t="n"/>
+      <c r="D12" s="46" t="inlineStr">
+        <is>
+          <t>Journal club 1 and debrief in one session: did the polarizer do what the menu says on this readout? Stick or pivot; decision in the group branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>Staff</t>
         </is>
       </c>
-      <c r="B12" s="55" t="inlineStr">
-        <is>
-          <t>Medium warmed, one vial per group at 13:00. Supervisor at the hood with each group for the thaw. Counting plates and MTT plates ready.</t>
-        </is>
-      </c>
-      <c r="C12" s="55" t="inlineStr">
-        <is>
-          <t>Cultures inspected 08:00. Counted staff suspension for the standard curves at 09:00. Plate reader 12:30 (column 1) and 14:30 (standard curve).</t>
-        </is>
-      </c>
-      <c r="D12" s="55" t="inlineStr">
-        <is>
-          <t>Freezing boxes in the -80. Plate reader 12:30 and 16:00. Collect all cultures at 17:00. Easter: vials to -140 on Fri 26 Mar; thaw backup RAW on Wed 31 Mar, split Fri 2 Apr: enough cells to plate four groups on Tue 6 Apr.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="45" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>Stock flasks counted per group at 12:30. Polarizers, vehicle and LPS at working concentration; plate maps checked before anyone pipettes.</t>
+        </is>
+      </c>
+      <c r="C13" s="55" t="inlineStr">
+        <is>
+          <t>Antibody panel, viability dye, fix/perm buffers, compensation beads. Nothing in the incubator but the stock flasks.</t>
+        </is>
+      </c>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>Escort the groups to the facility. Stock flasks: split, two or three backup vials to -80 per group, carried over the break by the staff. Easter: no course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="45" t="inlineStr">
         <is>
           <t>Resources</t>
         </is>
       </c>
-      <c r="B13" s="55" t="inlineStr">
+      <c r="B14" s="55" t="inlineStr">
         <is>
           <t>4 hoods HPL F27.2, one per group, available at all times. Cell counter.</t>
         </is>
       </c>
-      <c r="C13" s="55" t="inlineStr">
-        <is>
-          <t>4 hoods HPL F27.2, one per group, available at all times. Plate reader. Conference room HPL F22 for lectures and dry lab. FlowJo seats [TODO].</t>
-        </is>
-      </c>
-      <c r="D13" s="55" t="inlineStr">
-        <is>
-          <t>4 hoods HPL F27.2, one per group, available at all times. -80 box per group; Mr Frosty or equivalent [TODO: lab standard]. Plate reader. Conference room HPL F22 for lectures and dry lab.</t>
+      <c r="C14" s="55" t="inlineStr">
+        <is>
+          <t>4 hoods HPL F27.2, one per group, available at all times. Cooled centrifuge. Fridge. Conference room HPL F22 for lectures and dry lab.</t>
+        </is>
+      </c>
+      <c r="D14" s="55" t="inlineStr">
+        <is>
+          <t>Cytometer: 2 slots of 1.5 h [TODO: facility]. Conference room HPL F22 for lectures and dry lab. FlowJo seats [TODO].</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="10">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="B8:B11"/>
-    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D9:D11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1829,7 +1865,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1840,9 +1876,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
-        <is>
-          <t>Week 3: Exp 2, challenge and read out (Tue 6 - Fri 9 April 2027)</t>
+      <c r="A1" s="68" t="inlineStr">
+        <is>
+          <t>Week 3: polarize and challenge (Tue 6 - Fri 9 April 2027)</t>
         </is>
       </c>
       <c r="B1" s="32" t="n"/>
@@ -1891,7 +1927,7 @@
     <row r="4" ht="64" customHeight="1">
       <c r="A4" s="45" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="B4" s="48" t="inlineStr">
@@ -1899,217 +1935,245 @@
           <t>Your other lectures (not course time)</t>
         </is>
       </c>
-      <c r="C4" s="49" t="inlineStr">
-        <is>
-          <t>P05 Harvest: supernatants to -20 in aliquots for the ELISA, cells for flow cytometry (P08).</t>
-        </is>
-      </c>
-      <c r="D4" s="46" t="inlineStr">
-        <is>
-          <t>Journal club 2 (tbd): the peritoneal injury single-cell paper behind GSE186658 [TODO: paper]; one group presents, all read</t>
-        </is>
-      </c>
-      <c r="E4" s="54" t="inlineStr">
-        <is>
-          <t>FlowJo session: gating of your own data, export statistics (with the facility, tbd)</t>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
         </is>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="45" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B5" s="65" t="n"/>
-      <c r="C5" s="65" t="n"/>
-      <c r="D5" s="56" t="inlineStr">
-        <is>
-          <t>Cytometer slot, groups A+B: P08 Acquire [TODO: facility reservation]. Groups C+D: P06 ELISA, blocking and samples [TODO: timing against the protocol]; scRNA-seq part 2 during the incubations</t>
-        </is>
-      </c>
-      <c r="E5" s="65" t="n"/>
+      <c r="C5" s="49" t="inlineStr">
+        <is>
+          <t>P05 Challenge: your stimulus, optional inhibitor (TAK-242 1 h before, polymyxin B premixed), LPS on M(-) as everyone's control. Default: overnight, IL-6. Alternative: 6 h, TNF, harvest 15:00. Wet-lab goal: stimulate with inhibitor logic.</t>
+        </is>
+      </c>
+      <c r="D5" s="49" t="inlineStr">
+        <is>
+          <t>P05 Harvest (overnight groups): supernatants in aliquots, cells as RNA or protein lysate to the freezer</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t>ELISA analysis: standard curve, concentrations. Flow statistics from week 2 in R. scRNA-seq part 2 continued.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="64" customHeight="1">
       <c r="A6" s="45" t="inlineStr">
         <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="B6" s="66" t="n"/>
-      <c r="C6" s="66" t="n"/>
-      <c r="D6" s="66" t="n"/>
-      <c r="E6" s="66" t="n"/>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B6" s="65" t="n"/>
+      <c r="C6" s="65" t="n"/>
+      <c r="D6" s="49" t="inlineStr">
+        <is>
+          <t>P06 ELISA: blocking, standards, samples; dry lab in the incubations</t>
+        </is>
+      </c>
+      <c r="E6" s="65" t="n"/>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="45" t="inlineStr">
         <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="B7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="C7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="D7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="E7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="n"/>
+      <c r="C7" s="66" t="n"/>
+      <c r="D7" s="66" t="n"/>
+      <c r="E7" s="66" t="n"/>
     </row>
     <row r="8" ht="64" customHeight="1">
       <c r="A8" s="45" t="inlineStr">
         <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="B8" s="49" t="inlineStr">
-        <is>
-          <t>P02 Plate cells from the staff culture, spin the plate down, 2 h to adhere [TODO: confirm before the course that RAW cells adhere in 2 h after a spin]. Meanwhile P01 re-thaw your own vial (viability = Exp 1 readout). Then P05 Challenge overnight with LPS.</t>
-        </is>
-      </c>
-      <c r="C8" s="46" t="inlineStr">
-        <is>
-          <t>Lecture: single-cell transcriptomics for immunologists, what a signature score means (tbd)</t>
-        </is>
-      </c>
-      <c r="D8" s="56" t="inlineStr">
-        <is>
-          <t>Cytometer slot, groups C+D: P08 Acquire [TODO: facility reservation]. Groups A+B: P06 ELISA, blocking and samples [TODO: timing against the protocol]; scRNA-seq part 2 during the incubations</t>
-        </is>
-      </c>
-      <c r="E8" s="54" t="inlineStr">
-        <is>
-          <t>ELISA analysis: plate read if outstanding, standard curve, concentrations. Flow statistics in R. scRNA-seq part 2 continued. Poster: results so far</t>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
         </is>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1">
       <c r="A9" s="45" t="inlineStr">
         <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="B9" s="65" t="n"/>
-      <c r="C9" s="49" t="inlineStr">
-        <is>
-          <t>P08 Flow staining of the harvested cells, fix the stained cells (4 °C until acquisition). P06 Coat the ELISA plates with capture antibody, overnight at 4 °C [TODO: check the ELISA protocol]</t>
-        </is>
-      </c>
-      <c r="D9" s="65" t="n"/>
-      <c r="E9" s="65" t="n"/>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B9" s="49" t="inlineStr">
+        <is>
+          <t>P02 and P04: plate from your stock (carried over the break) with the chosen polarizer, own approach or the standard that worked. 96-well for supernatants, extra wells for lysates. Passage the stock.</t>
+        </is>
+      </c>
+      <c r="C9" s="46" t="inlineStr">
+        <is>
+          <t>Lecture: single-cell transcriptomics for immunologists, what a signature score means (tbd)</t>
+        </is>
+      </c>
+      <c r="D9" s="54" t="inlineStr">
+        <is>
+          <t>Dry lab during the ELISA incubations: the assay waits for 3.5 h in total, which is used to prepare the next steps and for dry lab (scRNA-seq part 2). The split of wet and dry lab may shift a little.</t>
+        </is>
+      </c>
+      <c r="E9" s="51" t="inlineStr">
+        <is>
+          <t>Poster: what the story has and what it is missing; week 4 plan agreed with your supervisor (repeat, add, or wrap up)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="64" customHeight="1">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="B10" s="66" t="n"/>
-      <c r="C10" s="65" t="n"/>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B10" s="65" t="n"/>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>Dry lab during the challenge: scRNA-seq part 2, signatures from the bulk RAW 264.7 dataset. TNF groups: harvest at 15:00, supernatants and lysates to the freezer.</t>
+        </is>
+      </c>
       <c r="D10" s="66" t="n"/>
-      <c r="E10" s="66" t="n"/>
+      <c r="E10" s="65" t="n"/>
     </row>
     <row r="11" ht="64" customHeight="1">
       <c r="A11" s="45" t="inlineStr">
         <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="B11" s="46" t="inlineStr">
-        <is>
-          <t>Cutting Edge Immunology Seminar 16:30-17:30 (tbd)</t>
-        </is>
-      </c>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B11" s="66" t="n"/>
       <c r="C11" s="66" t="n"/>
       <c r="D11" s="49" t="inlineStr">
         <is>
-          <t>ELISA: finish the detection steps or set the overnight step [TODO: protocol]</t>
-        </is>
-      </c>
-      <c r="E11" s="46" t="inlineStr">
-        <is>
-          <t>Debrief Exp 2: results, extension choices, rescue decisions</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
+          <t>P06 ELISA: detection and read-out; first look at the numbers. Passage the stock. Wet-lab goal: an ELISA from coating to concentration.</t>
+        </is>
+      </c>
+      <c r="E11" s="66" t="n"/>
+    </row>
+    <row r="12" ht="64" customHeight="1">
       <c r="A12" s="45" t="inlineStr">
         <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="B12" s="46" t="inlineStr">
+        <is>
+          <t>Cutting Edge Immunology Seminar 16:30-17:30 (tbd)</t>
+        </is>
+      </c>
+      <c r="C12" s="49" t="inlineStr">
+        <is>
+          <t>16:30: coat the ELISA plates with capture antibody, overnight at 4 °C (P06), 30 min at the bench</t>
+        </is>
+      </c>
+      <c r="D12" s="66" t="n"/>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>Debrief Exp 2: results and week 4 decisions</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="45" t="inlineStr">
+        <is>
           <t>Staff</t>
         </is>
       </c>
-      <c r="B12" s="55" t="inlineStr">
-        <is>
-          <t>Staff culture split Fri 2 Apr, counted at 12:30: enough cells to plate four groups. Plate maps checked before anyone pipettes. LPS aliquots at working concentration. Supervisor at the hood for the re-thaw.</t>
-        </is>
-      </c>
-      <c r="C12" s="55" t="inlineStr">
-        <is>
-          <t>Tubes labelled, -20 space for supernatants. Antibody panel, viability dye, fixation buffer. ELISA plates and capture antibody.</t>
-        </is>
-      </c>
-      <c r="D12" s="55" t="inlineStr">
-        <is>
-          <t>Escort the groups to the facility. ELISA reagents, plate reader booked.</t>
-        </is>
-      </c>
-      <c r="E12" s="55" t="inlineStr">
-        <is>
-          <t>FlowJo seats [TODO]. Plate reader. Staff culture kept for groups that need the rescue path (a repeat of Exp 2 in week 4).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="45" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>Stock flasks counted at 12:30. Polarizers, stimuli, inhibitors, LPS at working concentration. Plate maps checked.</t>
+        </is>
+      </c>
+      <c r="C13" s="55" t="inlineStr">
+        <is>
+          <t>Ligands, inhibitors and vehicle ready; -20 space and labelled tubes. Lysis buffers for RNA and protein.</t>
+        </is>
+      </c>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>ELISA reagents, plate reader booked. Flow on challenged cells only if a group found a slot in the regular booking.</t>
+        </is>
+      </c>
+      <c r="E13" s="55" t="inlineStr">
+        <is>
+          <t>Stock flasks: keep or freeze according to each group's week 4 plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="45" t="inlineStr">
         <is>
           <t>Resources</t>
         </is>
       </c>
-      <c r="B13" s="55" t="inlineStr">
+      <c r="B14" s="55" t="inlineStr">
         <is>
           <t>4 hoods HPL F27.2, one per group, available at all times. Plate centrifuge.</t>
         </is>
       </c>
-      <c r="C13" s="55" t="inlineStr">
-        <is>
-          <t>4 hoods HPL F27.2, one per group, available at all times. Cooled centrifuge. Fridge for the fixed cells and the coated plates. Conference room HPL F22 for lectures and dry lab.</t>
-        </is>
-      </c>
-      <c r="D13" s="55" t="inlineStr">
-        <is>
-          <t>Cytometer: 2 slots of 2 h [TODO: facility]. Plate reader (450 nm). 4 hoods HPL F27.2, one per group, available at all times. Conference room HPL F22 for lectures and dry lab.</t>
-        </is>
-      </c>
-      <c r="E13" s="55" t="inlineStr">
-        <is>
-          <t>Conference room HPL F22 for lectures and dry lab. FlowJo seats [TODO]. Plate reader. 4 hoods HPL F27.2, one per group, available at all times.</t>
+      <c r="C14" s="55" t="inlineStr">
+        <is>
+          <t>4 hoods HPL F27.2, one per group, available at all times. Conference room HPL F22 for lectures and dry lab.</t>
+        </is>
+      </c>
+      <c r="D14" s="55" t="inlineStr">
+        <is>
+          <t>Plate reader (450 nm). 4 hoods HPL F27.2, one per group, available at all times. Conference room HPL F22 for lectures and dry lab.</t>
+        </is>
+      </c>
+      <c r="E14" s="55" t="inlineStr">
+        <is>
+          <t>Conference room HPL F22 for lectures and dry lab. 4 hoods HPL F27.2, one per group, available at all times.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
+    <mergeCell ref="D9:D10"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="E4:E6"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="B9:B11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C9:C11"/>
-    <mergeCell ref="C4:C6"/>
-    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="E5:E7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E9:E11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2121,7 +2185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2132,9 +2196,9 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="63" t="inlineStr">
-        <is>
-          <t>Week 4: extensions, poster, presentations (Tue 13 - Fri 16 April 2027)</t>
+      <c r="A1" s="68" t="inlineStr">
+        <is>
+          <t>Week 4: close the story (Tue 13 - Fri 16 April 2027)</t>
         </is>
       </c>
       <c r="B1" s="32" t="n"/>
@@ -2183,7 +2247,7 @@
     <row r="4" ht="64" customHeight="1">
       <c r="A4" s="45" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="B4" s="48" t="inlineStr">
@@ -2191,208 +2255,223 @@
           <t>Your other lectures (not course time)</t>
         </is>
       </c>
-      <c r="C4" s="46" t="inlineStr">
-        <is>
-          <t>Lecture: scientific writing, from data to argument, poster structure, figure design, honest limits (tbd)</t>
-        </is>
-      </c>
-      <c r="D4" s="51" t="inlineStr">
-        <is>
-          <t>Poster production with your supervisor: final figures and legends</t>
-        </is>
-      </c>
-      <c r="E4" s="54" t="inlineStr">
-        <is>
-          <t>Lab clean-up; notebook and group branch finalised</t>
+      <c r="C4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
+        </is>
+      </c>
+      <c r="D4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
+        </is>
+      </c>
+      <c r="E4" s="48" t="inlineStr">
+        <is>
+          <t>Self-study: reading for the day, notebook, group branch</t>
         </is>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1">
       <c r="A5" s="45" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="B5" s="65" t="n"/>
       <c r="C5" s="50" t="inlineStr">
         <is>
-          <t>Extension, continued, or rescue path: harvest, flow staining, ELISA</t>
-        </is>
-      </c>
-      <c r="D5" s="65" t="n"/>
-      <c r="E5" s="66" t="n"/>
+          <t>Optional harvest and ELISA for groups at the bench; otherwise poster: figures and legends</t>
+        </is>
+      </c>
+      <c r="D5" s="51" t="inlineStr">
+        <is>
+          <t>Wrap up: code, figures and poster, with your supervisor. Print when ready (signprint.ch); the PDF goes to the group branch first</t>
+        </is>
+      </c>
+      <c r="E5" s="54" t="inlineStr">
+        <is>
+          <t>Lab cleaning</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="64" customHeight="1">
       <c r="A6" s="45" t="inlineStr">
         <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="B6" s="66" t="n"/>
-      <c r="C6" s="66" t="n"/>
-      <c r="D6" s="66" t="n"/>
-      <c r="E6" s="46" t="inlineStr">
-        <is>
-          <t>Feedback round with the teaching staff; course evaluation</t>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="B6" s="65" t="n"/>
+      <c r="C6" s="65" t="n"/>
+      <c r="D6" s="65" t="n"/>
+      <c r="E6" s="54" t="inlineStr">
+        <is>
+          <t>Finish the group branch; poster pickup, self-service</t>
         </is>
       </c>
     </row>
     <row r="7" ht="64" customHeight="1">
       <c r="A7" s="45" t="inlineStr">
         <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="B7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="C7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="D7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
-      <c r="E7" s="48" t="inlineStr">
-        <is>
-          <t>Lunch</t>
-        </is>
-      </c>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B7" s="66" t="n"/>
+      <c r="C7" s="66" t="n"/>
+      <c r="D7" s="66" t="n"/>
+      <c r="E7" s="66" t="n"/>
     </row>
     <row r="8" ht="64" customHeight="1">
       <c r="A8" s="45" t="inlineStr">
         <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="B8" s="50" t="inlineStr">
-        <is>
-          <t>Extension of your choice (bench steps), or rescue path: repeat Exp 2 (plate, spin, 2 h, LPS challenge overnight)</t>
-        </is>
-      </c>
-      <c r="C8" s="51" t="inlineStr">
-        <is>
-          <t>Dry lab: analysis of Exp 2 and the extension, scRNA-seq part 3, score the tissue macrophages. Poster: figures and legends</t>
-        </is>
-      </c>
-      <c r="D8" s="51" t="inlineStr">
-        <is>
-          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch</t>
-        </is>
-      </c>
-      <c r="E8" s="46" t="inlineStr">
-        <is>
-          <t>Poster presentations and discussion; prize</t>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="C8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="D8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="E8" s="48" t="inlineStr">
+        <is>
+          <t>Lunch</t>
         </is>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1">
       <c r="A9" s="45" t="inlineStr">
         <is>
-          <t>14:00</t>
-        </is>
-      </c>
-      <c r="B9" s="65" t="n"/>
-      <c r="C9" s="65" t="n"/>
-      <c r="D9" s="46" t="inlineStr">
-        <is>
-          <t>Recap and Q&amp;A (tbd): the course in one hour, then open questions with the teaching staff</t>
-        </is>
-      </c>
-      <c r="E9" s="65" t="n"/>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="B9" s="50" t="inlineStr">
+        <is>
+          <t>Optional, as agreed on 9 April: repeat the polarization or the challenge, or a third experiment. Or dry lab: finish the in silico part and the poster. Never at the cost of wrapping up.</t>
+        </is>
+      </c>
+      <c r="C9" s="51" t="inlineStr">
+        <is>
+          <t>Wrap up: code, figures and poster; scRNA-seq part 3, score the tissue macrophages</t>
+        </is>
+      </c>
+      <c r="D9" s="51" t="inlineStr">
+        <is>
+          <t>Wrap up, continued: code, figures, poster, group branch. Stock flask frozen or discarded.</t>
+        </is>
+      </c>
+      <c r="E9" s="46" t="inlineStr">
+        <is>
+          <t>Written exam, individual [TODO: duration and room]</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="64" customHeight="1">
       <c r="A10" s="45" t="inlineStr">
         <is>
-          <t>15:00</t>
-        </is>
-      </c>
-      <c r="B10" s="66" t="n"/>
-      <c r="C10" s="66" t="n"/>
-      <c r="D10" s="48" t="inlineStr">
-        <is>
-          <t>Free: extension analysis, notebook, group branch</t>
-        </is>
-      </c>
-      <c r="E10" s="66" t="n"/>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="B10" s="65" t="n"/>
+      <c r="C10" s="65" t="n"/>
+      <c r="D10" s="65" t="n"/>
+      <c r="E10" s="46" t="inlineStr">
+        <is>
+          <t>Poster session: presentations and discussion; prize</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="64" customHeight="1">
       <c r="A11" s="45" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="B11" s="66" t="n"/>
+      <c r="C11" s="66" t="n"/>
+      <c r="D11" s="65" t="n"/>
+      <c r="E11" s="66" t="n"/>
+    </row>
+    <row r="12" ht="64" customHeight="1">
+      <c r="A12" s="45" t="inlineStr">
+        <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="B11" s="46" t="inlineStr">
+      <c r="B12" s="46" t="inlineStr">
         <is>
           <t>Cutting Edge Immunology Seminar 16:30-17:30 (tbd)</t>
         </is>
       </c>
-      <c r="C11" s="46" t="inlineStr">
-        <is>
-          <t>Failure round: each group presents one thing that went wrong and what it taught them</t>
-        </is>
-      </c>
-      <c r="D11" s="66" t="n"/>
-      <c r="E11" s="46" t="inlineStr">
-        <is>
-          <t>Apéro</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="45" t="inlineStr">
+      <c r="C12" s="46" t="inlineStr">
+        <is>
+          <t>Publish or perish: a critical discussion on scientific integrity and output metrics</t>
+        </is>
+      </c>
+      <c r="D12" s="66" t="n"/>
+      <c r="E12" s="46" t="inlineStr">
+        <is>
+          <t>Open 360° feedback round: closes the poster session and opens the apéro</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="45" t="inlineStr">
         <is>
           <t>Staff</t>
         </is>
       </c>
-      <c r="B12" s="55" t="inlineStr">
-        <is>
-          <t>Reagents for the extensions agreed on Fri 9 Apr. Staff culture ready for rescue groups to plate.</t>
-        </is>
-      </c>
-      <c r="C12" s="55" t="inlineStr">
-        <is>
-          <t>Poster template distributed, printing booked [TODO: printer]. Rescue groups: cytometer slot [TODO: facility], ELISA Wed, result on the poster by Thursday.</t>
-        </is>
-      </c>
-      <c r="D12" s="55" t="inlineStr">
-        <is>
-          <t>Posters printed Thu after 14:00 [TODO: printer].</t>
-        </is>
-      </c>
-      <c r="E12" s="55" t="inlineStr">
-        <is>
-          <t>Jury, prize, evaluation form, clean-up checklist. Apéro ordered [TODO: catering].</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="64" customHeight="1">
-      <c r="A13" s="45" t="inlineStr">
+      <c r="B13" s="55" t="inlineStr">
+        <is>
+          <t>Reagents for the agreed repeats or extensions. Stock flasks for the groups that plate.</t>
+        </is>
+      </c>
+      <c r="C13" s="55" t="inlineStr">
+        <is>
+          <t>Poster template distributed. Plate reader for the groups that ran an ELISA.</t>
+        </is>
+      </c>
+      <c r="D13" s="55" t="inlineStr">
+        <is>
+          <t>Poster boards ready. Exam papers printed. Course evaluation goes out as a written survey.</t>
+        </is>
+      </c>
+      <c r="E13" s="55" t="inlineStr">
+        <is>
+          <t>Exam papers, jury, prize, clean-up checklist. Apéro ordered [TODO: catering]; evaluation survey sent after the course.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="45" t="inlineStr">
         <is>
           <t>Resources</t>
         </is>
       </c>
-      <c r="B13" s="55" t="inlineStr">
-        <is>
-          <t>4 hoods HPL F27.2, one per group, available at all times. Extension-specific instruments as agreed.</t>
-        </is>
-      </c>
-      <c r="C13" s="55" t="inlineStr">
+      <c r="B14" s="55" t="inlineStr">
+        <is>
+          <t>4 hoods HPL F27.2, one per group, available at all times. Extension-specific instruments as agreed. Conference room HPL F22 for lectures and dry lab.</t>
+        </is>
+      </c>
+      <c r="C14" s="55" t="inlineStr">
         <is>
           <t>4 hoods HPL F27.2, one per group, available at all times. Conference room HPL F22 for lectures and dry lab.</t>
         </is>
       </c>
-      <c r="D13" s="55" t="inlineStr">
-        <is>
-          <t>Conference room HPL F22 for lectures and dry lab. Printer [TODO]. Poster boards.</t>
-        </is>
-      </c>
-      <c r="E13" s="55" t="inlineStr">
+      <c r="D14" s="55" t="inlineStr">
+        <is>
+          <t>Conference room HPL F22 for lectures and dry lab. Poster boards.</t>
+        </is>
+      </c>
+      <c r="E14" s="55" t="inlineStr">
         <is>
           <t>Conference room HPL F22 for lectures and dry lab. Apéro room [TODO: catering].</t>
         </is>
@@ -2400,16 +2479,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
-    <mergeCell ref="D4:D6"/>
-    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="D9:D12"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="D5:D7"/>
+    <mergeCell ref="B4:B7"/>
+    <mergeCell ref="B9:B11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C5:C7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="C9:C11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Days 1 and 2: introductory lecture, lab and biosafety session, supervisor round, git afternoon
Thursday: welcome and introductory lecture 09:00-10:15, working in the lab
and biosafety with Q&A and the signing of the safety sheet 10:30-12:00,
introduction of the supervisors and group formation 13:00, planning as
before. Friday afternoon 13:00-17:00: git and RStudio from scratch, ending
with the ELISA script run and one line pushed to the group branch. The
February email is an open item; the plan assumes some will not have read it.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,6 +507,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1240,12 +1246,12 @@
       <c r="D4" s="41" t="n"/>
       <c r="E4" s="46" t="inlineStr">
         <is>
-          <t>Welcome, lecture, group formation; the pathway drawing and the menu choices</t>
+          <t>Welcome and introductory lecture; lab and biosafety; supervisors and groups; the pathway drawing and the menu choices</t>
         </is>
       </c>
       <c r="F4" s="47" t="inlineStr">
         <is>
-          <t>Hands-on cell culture; thaw and seed the group's stock flask; dry lab setup; plan committed</t>
+          <t>Hands-on cell culture; thaw and seed the group's stock flask; git and RStudio from scratch; plan committed</t>
         </is>
       </c>
     </row>
@@ -1395,7 +1401,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="70" t="inlineStr">
+      <c r="A1" s="72" t="inlineStr">
         <is>
           <t>Week 1: orientation (Thu 18 - Fri 19 March 2027)</t>
         </is>
@@ -1454,7 +1460,7 @@
       </c>
       <c r="B5" s="46" t="inlineStr">
         <is>
-          <t>Welcome and safety briefing (Tea Kocijan)</t>
+          <t>Welcome address and introductory lecture: macrophages, why they matter, why we do what we do (Joel Zindel), 09:00-10:15</t>
         </is>
       </c>
       <c r="C5" s="47" t="inlineStr">
@@ -1469,11 +1475,7 @@
           <t>10:00</t>
         </is>
       </c>
-      <c r="B6" s="46" t="inlineStr">
-        <is>
-          <t>Lecture: tissue macrophages and nomenclature (Joel Zindel)</t>
-        </is>
-      </c>
+      <c r="B6" s="66" t="n"/>
       <c r="C6" s="65" t="n"/>
     </row>
     <row r="7" ht="64" customHeight="1">
@@ -1482,7 +1484,11 @@
           <t>11:00</t>
         </is>
       </c>
-      <c r="B7" s="66" t="n"/>
+      <c r="B7" s="46" t="inlineStr">
+        <is>
+          <t>Working in the lab and biosafety (Tea Kocijan), 10:30-12:00: Q&amp;A, then the safety sheet is signed</t>
+        </is>
+      </c>
       <c r="C7" s="66" t="n"/>
     </row>
     <row r="8" ht="64" customHeight="1">
@@ -1510,12 +1516,12 @@
       </c>
       <c r="B9" s="46" t="inlineStr">
         <is>
-          <t>Group formation</t>
+          <t>Introduction of the supervisors (what they do and why) and group formation</t>
         </is>
       </c>
       <c r="C9" s="54" t="inlineStr">
         <is>
-          <t>Dry lab setup: clone the course repository, build the environment with your chatty, run the ELISA template on example data. Group plan (the drawing and your menu choices) committed to the group branch at 17:00.</t>
+          <t>Working with git and RStudio, step by step with the supervisors: GitHub account, install R, RStudio and Git if you did not at home, token, clone the course repository from RStudio, switch to your group's branch, open the ELISA script and run it, push one line to the branch. Then build the rest of the environment with your chatty. Group plan (the drawing and your menu choices) committed to the group branch at 17:00.</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1533,7 @@
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisors: hand-draw the pathway you will test (ligand, receptor, output, how an inhibitor proves it, where the polarizer acts), pick your polarizer, stimulus and cytokine (P04, P05, P06). Read P01, P02 and P08 for Friday and Tuesday.</t>
+          <t>Experiment planning with your supervisors: hand-draw the pathway you will test (ligand, receptor, output, how an inhibitor proves it, where the polarizer acts), pick your polarizer, stimulus and cytokine (P04, P05, P06) and your extension. Read P01, P02 and P08 for Friday and Tuesday.</t>
         </is>
       </c>
       <c r="C10" s="65" t="n"/>
@@ -1558,12 +1564,12 @@
       </c>
       <c r="B13" s="55" t="inlineStr">
         <is>
-          <t>Rooms, safety officer. Groups formed at 13:00; supervisors sit with their group from then on.</t>
+          <t>Rooms, safety officer. Signed safety sheets collected at 12:00. Supervisors sit with their group from 14:00.</t>
         </is>
       </c>
       <c r="C13" s="55" t="inlineStr">
         <is>
-          <t>One low-passage vial per group. Supervisors carry the stock flasks over the weekend and the break: split every 2 to 3 days, course passage counted from this thaw. Dry lab: unblock installs; fallback environment ready [TODO]. Collect the plans at 17:00.</t>
+          <t>One low-passage vial per group. Supervisors carry the stock flasks over the weekend and the break: split every 2 to 3 days, course passage counted from this thaw. Afternoon: one supervisor per two laptops; the 08:00 slot is the installation help desk for latecomers. Collect the plans at 17:00.</t>
         </is>
       </c>
     </row>
@@ -1590,7 +1596,7 @@
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="B10:B12"/>
     <mergeCell ref="C5:C7"/>
-    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="B5:B6"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1613,7 +1619,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="70" t="inlineStr">
+      <c r="A1" s="72" t="inlineStr">
         <is>
           <t>Week 2: polarize and characterize (Tue 23 - Thu 25 March 2027)</t>
         </is>
@@ -1882,7 +1888,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="70" t="inlineStr">
+      <c r="A1" s="72" t="inlineStr">
         <is>
           <t>Week 3: polarize and challenge (Tue 6 - Fri 9 April 2027)</t>
         </is>
@@ -2202,7 +2208,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="70" t="inlineStr">
+      <c r="A1" s="72" t="inlineStr">
         <is>
           <t>Week 4: close the story (Tue 13 - Fri 16 April 2027)</t>
         </is>

</xml_diff>

<commit_message>
Notebooks folder: one text file per person, first commit "hello world" on Friday of week 1
The git smoke test is the first notebook entry: new text file in RStudio,
saved under a name of your choice in notebooks/, committed as "hello world",
pushed to the group branch. README Section 3 points there for the lab
notebook; the folder page carries the rules (one file per person, pull and
push daily, support commits).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,6 +507,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1401,7 +1404,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="72" t="inlineStr">
+      <c r="A1" s="73" t="inlineStr">
         <is>
           <t>Week 1: orientation (Thu 18 - Fri 19 March 2027)</t>
         </is>
@@ -1521,7 +1524,7 @@
       </c>
       <c r="C9" s="54" t="inlineStr">
         <is>
-          <t>Working with git and RStudio, step by step with the supervisors: GitHub account, install R, RStudio and Git if you did not at home, token, clone the course repository from RStudio, switch to your group's branch, open the ELISA script and run it, push one line to the branch. Then build the rest of the environment with your chatty. Group plan (the drawing and your menu choices) committed to the group branch at 17:00.</t>
+          <t>Working with git and RStudio, step by step with the supervisors: GitHub account, install R, RStudio and Git if you did not at home, token, clone the course repository from RStudio, switch to your group's branch, open the ELISA script and run it. Then the first commit: a new text file in notebooks/ with your first notes, saved under a name you like, committed as "hello world" and pushed to your branch. Then the rest of the environment with your chatty. Group plan (the drawing and your menu choices) committed to the group branch at 17:00.</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1622,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="72" t="inlineStr">
+      <c r="A1" s="73" t="inlineStr">
         <is>
           <t>Week 2: polarize and characterize (Tue 23 - Thu 25 March 2027)</t>
         </is>
@@ -1888,7 +1891,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="72" t="inlineStr">
+      <c r="A1" s="73" t="inlineStr">
         <is>
           <t>Week 3: polarize and challenge (Tue 6 - Fri 9 April 2027)</t>
         </is>
@@ -2208,7 +2211,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="72" t="inlineStr">
+      <c r="A1" s="73" t="inlineStr">
         <is>
           <t>Week 4: close the story (Tue 13 - Fri 16 April 2027)</t>
         </is>

</xml_diff>

<commit_message>
Merge core and optional experiments into Section 5 with three experiments
README: Sections 5 ("Core experiments") and 6 ("Optional experiments") become one
section, "5. Experiments", with Experiment 1: Polarization (wet lab, week 2),
Experiment 2: Comparison in vitro versus in vivo polarization (dry lab, weeks 2 to 4)
and Experiment 3: Challenge with danger signals (wet lab, week 3). The extensions
table becomes the subsection "Extensions" at the end of Section 5; Assessment,
Writing and Safety are renumbered 6 to 8.

Experiment numbers are renumbered everywhere else (llms.txt, protocol headers and
index, background, schedule builder legend and labels, notebooks and poster
section references), and the schedule, figures and companion are regenerated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,6 +507,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -965,12 +968,12 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>EXP2</t>
+          <t>EXP3</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Wet lab Exp 2: polarize and challenge (plate, stimulate, harvest, ELISA)</t>
+          <t>Wet lab Exp 3: polarize and challenge (plate, stimulate, harvest, ELISA)</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1081,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Exp 1 (week 2): polarize and characterize. Plate from the group's stock with the polarizer in the seeding suspension, vehicle and LPS controls beside it; harvest, stain, acquire; FlowJo; decide to stick or pivot before the break. Exp 2 (week 3): polarize and challenge. Plate with the polarizer on Tuesday, challenge on Wednesday with the group's stimulus and optional inhibitor (LPS on M(-) shared by all), overnight with an IL-6 readout by default or 6 h with TNF; ELISA on Thursday. Week 4: repeat, add, or wrap up. Menus in P04 and P05. Protocol IDs (P01...) refer to protocols/ in the course repository.</t>
+          <t>Exp 1 (week 2): polarize and characterize. Plate from the group's stock with the polarizer in the seeding suspension, vehicle and LPS controls beside it; harvest, stain, acquire; FlowJo; decide to stick or pivot before the break. Exp 2 (dry lab, weeks 2 to 4): comparison of in vitro versus in vivo polarization, see the Dry lab row. Exp 3 (week 3): polarize and challenge. Plate with the polarizer on Tuesday, challenge on Wednesday with the group's stimulus and optional inhibitor (LPS on M(-) shared by all), overnight with an IL-6 readout by default or 6 h with TNF; ELISA on Thursday. Week 4: repeat, add, or wrap up. Menus in P04 and P05. Protocol IDs (P01...) refer to protocols/ in the course repository.</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1093,7 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Week 1: environment and templates. Week 2: scRNA-seq part 1 (QC) in the afternoon dry-lab slots, FlowJo on the own data. Week 3: scRNA-seq part 2 (signatures from the bulk RAW 264.7 dataset) during the challenge and the ELISA incubations, own ELISA data on Friday. Week 4: scRNA-seq part 3 (scoring of the tissue macrophages), wrap up of code, figures and poster.</t>
+          <t>Week 1: environment and templates. Exp 2, the in silico comparison, runs through weeks 2 to 4. Week 2: scRNA-seq part 1 (QC) in the afternoon dry-lab slots, FlowJo on the own data. Week 3: scRNA-seq part 2 (signatures from the bulk RAW 264.7 dataset) during the challenge and the ELISA incubations, own ELISA data on Friday. Week 4: scRNA-seq part 3 (scoring of the tissue macrophages), wrap up of code, figures and poster.</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1354,7 @@
       </c>
       <c r="C8" s="50" t="inlineStr">
         <is>
-          <t>Morning: other lectures. 13:00 optional repeat, third experiment, or dry lab</t>
+          <t>Morning: other lectures. 13:00 optional repeat, further experiment, or dry lab</t>
         </is>
       </c>
       <c r="D8" s="51" t="inlineStr">
@@ -1404,7 +1407,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="73" t="inlineStr">
+      <c r="A1" s="74" t="inlineStr">
         <is>
           <t>Week 1: orientation (Thu 18 - Fri 19 March 2027)</t>
         </is>
@@ -1622,7 +1625,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="73" t="inlineStr">
+      <c r="A1" s="74" t="inlineStr">
         <is>
           <t>Week 2: polarize and characterize (Tue 23 - Thu 25 March 2027)</t>
         </is>
@@ -1891,7 +1894,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="73" t="inlineStr">
+      <c r="A1" s="74" t="inlineStr">
         <is>
           <t>Week 3: polarize and challenge (Tue 6 - Fri 9 April 2027)</t>
         </is>
@@ -2118,7 +2121,7 @@
       <c r="D12" s="66" t="n"/>
       <c r="E12" s="46" t="inlineStr">
         <is>
-          <t>Debrief Exp 2: results and week 4 decisions</t>
+          <t>Debrief Exp 3: results and week 4 decisions</t>
         </is>
       </c>
     </row>
@@ -2211,7 +2214,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="73" t="inlineStr">
+      <c r="A1" s="74" t="inlineStr">
         <is>
           <t>Week 4: close the story (Tue 13 - Fri 16 April 2027)</t>
         </is>
@@ -2370,7 +2373,7 @@
       </c>
       <c r="B9" s="50" t="inlineStr">
         <is>
-          <t>Optional, as agreed on 9 April: repeat the polarization or the challenge, or a third experiment. Or dry lab: finish the in silico part and the poster. Never at the cost of wrapping up.</t>
+          <t>Optional, as agreed on 9 April: repeat the polarization or the challenge, or a further experiment. Or dry lab: finish the in silico part and the poster. Never at the cost of wrapping up.</t>
         </is>
       </c>
       <c r="C9" s="51" t="inlineStr">

</xml_diff>

<commit_message>
Say AI tool instead of chatty everywhere
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -335,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -507,6 +507,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1407,7 +1410,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>Week 1: orientation (Thu 18 - Fri 19 March 2027)</t>
         </is>
@@ -1527,7 +1530,7 @@
       </c>
       <c r="C9" s="54" t="inlineStr">
         <is>
-          <t>Working with git and RStudio, step by step with the supervisors: GitHub account, install R, RStudio and Git if you did not at home, token, clone the course repository from RStudio, switch to your group's branch, open the ELISA script and run it. Then the first commit: a new text file in notebooks/ with your first notes, saved under a name you like, committed as "hello world" and pushed to your branch. Then the rest of the environment with your chatty. Group plan (the drawing and your menu choices) committed to the group branch at 17:00.</t>
+          <t>Working with git and RStudio, step by step with the supervisors: GitHub account, install R, RStudio and Git if you did not at home, token, clone the course repository from RStudio, switch to your group's branch, open the ELISA script and run it. Then the first commit: a new text file in notebooks/ with your first notes, saved under a name you like, committed as "hello world" and pushed to your branch. Then the rest of the environment with your AI tool. Group plan (the drawing and your menu choices) committed to the group branch at 17:00.</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1628,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>Week 2: polarize and characterize (Tue 23 - Thu 25 March 2027)</t>
         </is>
@@ -1894,7 +1897,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>Week 3: polarize and challenge (Tue 6 - Fri 9 April 2027)</t>
         </is>
@@ -2214,7 +2217,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="74" t="inlineStr">
+      <c r="A1" s="75" t="inlineStr">
         <is>
           <t>Week 4: close the story (Tue 13 - Fri 16 April 2027)</t>
         </is>

</xml_diff>

<commit_message>
Protocols: five core protocols (C1-C5), extensions X01-X05, staff S01; boxed times and GitHub callouts
- P01 and P02 merged into C1 RAW 264.7 culture: thaw, split, seed
- P04, P08, P05, P06 become C2-C5 in course order; P07 Griess and P09 MTT become X04 and X05; P03 freeze becomes staff protocol S01
- All references updated (script, llms.txt, safety, code, Gantt workbook and builder)
- Formatting convention in the template: incubations and spins bold and boxed, callouts as top-level GitHub alerts
- build_companion picks up C*, X* and S* files

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -920,6 +920,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1028,6 +1029,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
@@ -1084,7 +1086,7 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Exp 1 (week 2): polarize and characterize. Plate from the group's stock with the polarizer in the seeding suspension, vehicle and LPS controls beside it; harvest, stain, acquire; FlowJo; decide to stick or pivot before the break. Exp 2 (dry lab, weeks 2 to 4): comparison of in vitro versus in vivo polarization, see the Dry lab row. Exp 3 (week 3): polarize and challenge. Plate with the polarizer on Tuesday, challenge on Wednesday with the group's stimulus and optional inhibitor (LPS on M(-) shared by all), overnight with an IL-6 readout by default or 6 h with TNF; ELISA on Thursday. Week 4: repeat, add, or wrap up. Menus in P04 and P05. Protocol IDs (P01...) refer to protocols/ in the course repository.</t>
+          <t>Exp 1 (week 2): polarize and characterize. Plate from the group's stock with the polarizer in the seeding suspension, vehicle and LPS controls beside it; harvest, stain, acquire; FlowJo; decide to stick or pivot before the break. Exp 2 (dry lab, weeks 2 to 4): comparison of in vitro versus in vivo polarization, see the Dry lab row. Exp 3 (week 3): polarize and challenge. Plate with the polarizer on Tuesday, challenge on Wednesday with the group's stimulus and optional inhibitor (LPS on M(-) shared by all), overnight with an IL-6 readout by default or 6 h with TNF; ELISA on Thursday. Week 4: repeat, add, or wrap up. Menus in C2 and C4. Protocol IDs (C1...) refer to protocols/ in the course repository.</t>
         </is>
       </c>
     </row>
@@ -1124,6 +1126,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
@@ -1216,6 +1219,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="44" t="inlineStr"/>
       <c r="B3" s="45" t="inlineStr">
@@ -1376,6 +1380,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1474,7 +1479,7 @@
       </c>
       <c r="C5" s="47" t="inlineStr">
         <is>
-          <t>Hands-on cell culture with the staff culture: hood and sterile technique, microscope, P02 scrape, count, split and seed, cell counter. Then P01: thaw and seed your group's stock flask (course passage 0). Lab tour.</t>
+          <t>Hands-on cell culture with the staff culture: hood and sterile technique, microscope, C1 scrape, count, split and seed, cell counter. Then C1: thaw and seed your group's stock flask (course passage 0). Lab tour.</t>
         </is>
       </c>
     </row>
@@ -1542,7 +1547,7 @@
       </c>
       <c r="B10" s="54" t="inlineStr">
         <is>
-          <t>Experiment planning with your supervisors: hand-draw the pathway you will test (ligand, receptor, output, how an inhibitor proves it, where the polarizer acts), pick your polarizer, stimulus and cytokine (P04, P05, P06) and your extension. Read P01, P02 and P08 for Friday and Tuesday.</t>
+          <t>Experiment planning with your supervisors: hand-draw the pathway you will test (ligand, receptor, output, how an inhibitor proves it, where the polarizer acts), pick your polarizer, stimulus and cytokine (C2, C4, C5) and your extension. Read C1 and C3 for Friday and Tuesday.</t>
         </is>
       </c>
       <c r="C10" s="65" t="n"/>
@@ -1705,7 +1710,7 @@
       </c>
       <c r="D5" s="56" t="inlineStr">
         <is>
-          <t>P08 Acquisition at the facility, two batches of 1.5 h, two groups each [TODO: reservation]</t>
+          <t>C3 Acquisition at the facility, two batches of 1.5 h, two groups each [TODO: reservation]</t>
         </is>
       </c>
     </row>
@@ -1718,7 +1723,7 @@
       <c r="B6" s="65" t="n"/>
       <c r="C6" s="47" t="inlineStr">
         <is>
-          <t>P08 Harvest the adherent cells, count, viability dye, Fc block, surface stain</t>
+          <t>C3 Harvest the adherent cells, count, viability dye, Fc block, surface stain</t>
         </is>
       </c>
       <c r="D6" s="65" t="n"/>
@@ -1763,12 +1768,12 @@
       </c>
       <c r="B9" s="47" t="inlineStr">
         <is>
-          <t>P02 and P04: plate cells from your stock with the polarizer already in the seeding suspension. Vehicle control, M(pol) and LPS control on the flow plate (6- or 12-well). Plate-and-polarize in one step, about 19 h. Wet-lab goal: plate at a defined density with a stimulus.</t>
+          <t>C1 and C2: plate cells from your stock with the polarizer already in the seeding suspension. Vehicle control, M(pol) and LPS control on the flow plate (6- or 12-well). Plate-and-polarize in one step, about 19 h. Wet-lab goal: plate at a defined density with a stimulus.</t>
         </is>
       </c>
       <c r="C9" s="47" t="inlineStr">
         <is>
-          <t>P08 continued: optional Arg1 fix and perm, fix, store at 4 °C until acquisition. Wet-lab goal: harvest, staining, fixation. Staining plan and FMOs in the notebook.</t>
+          <t>C3 continued: optional Arg1 fix and perm, fix, store at 4 °C until acquisition. Wet-lab goal: harvest, staining, fixation. Staining plan and FMOs in the notebook.</t>
         </is>
       </c>
       <c r="D9" s="56" t="inlineStr">
@@ -1981,12 +1986,12 @@
       <c r="B5" s="65" t="n"/>
       <c r="C5" s="49" t="inlineStr">
         <is>
-          <t>P05 Challenge: your stimulus, optional inhibitor (TAK-242 1 h before, polymyxin B premixed), LPS on M(-) as everyone's control. Default: overnight, IL-6. Alternative: 6 h, TNF, harvest 15:00. Wet-lab goal: stimulate with inhibitor logic.</t>
+          <t>C4 Challenge: your stimulus, optional inhibitor (TAK-242 1 h before, polymyxin B premixed), LPS on M(-) as everyone's control. Default: overnight, IL-6. Alternative: 6 h, TNF, harvest 15:00. Wet-lab goal: stimulate with inhibitor logic.</t>
         </is>
       </c>
       <c r="D5" s="49" t="inlineStr">
         <is>
-          <t>P05 Harvest (overnight groups): supernatants in aliquots, cells as RNA or protein lysate to the freezer</t>
+          <t>C4 Harvest (overnight groups): supernatants in aliquots, cells as RNA or protein lysate to the freezer</t>
         </is>
       </c>
       <c r="E5" s="54" t="inlineStr">
@@ -2005,7 +2010,7 @@
       <c r="C6" s="65" t="n"/>
       <c r="D6" s="49" t="inlineStr">
         <is>
-          <t>P06 ELISA: blocking, standards, samples; dry lab in the incubations</t>
+          <t>C5 ELISA: blocking, standards, samples; dry lab in the incubations</t>
         </is>
       </c>
       <c r="E6" s="65" t="n"/>
@@ -2056,7 +2061,7 @@
       </c>
       <c r="B9" s="49" t="inlineStr">
         <is>
-          <t>P02 and P04: plate from your stock (carried over the break) with the chosen polarizer, own approach or the standard that worked. 96-well for supernatants, extra wells for lysates. Passage the stock.</t>
+          <t>C1 and C2: plate from your stock (carried over the break) with the chosen polarizer, own approach or the standard that worked. 96-well for supernatants, extra wells for lysates. Passage the stock.</t>
         </is>
       </c>
       <c r="C9" s="46" t="inlineStr">
@@ -2100,7 +2105,7 @@
       <c r="C11" s="66" t="n"/>
       <c r="D11" s="49" t="inlineStr">
         <is>
-          <t>P06 ELISA: detection and read-out; first look at the numbers. Passage the stock. Wet-lab goal: an ELISA from coating to concentration.</t>
+          <t>C5 ELISA: detection and read-out; first look at the numbers. Passage the stock. Wet-lab goal: an ELISA from coating to concentration.</t>
         </is>
       </c>
       <c r="E11" s="66" t="n"/>
@@ -2118,7 +2123,7 @@
       </c>
       <c r="C12" s="49" t="inlineStr">
         <is>
-          <t>16:30: coat the ELISA plates with capture antibody, overnight at 4 °C (P06), 30 min at the bench</t>
+          <t>16:30: coat the ELISA plates with capture antibody, overnight at 4 °C (C5), 30 min at the bench</t>
         </is>
       </c>
       <c r="D12" s="66" t="n"/>

</xml_diff>

<commit_message>
Admission sheet (safety and data) replaces the safety sheet; README Section 9 Data
- safety/README.md: new section 3 Your data (data belong to the lab, rights transferred to ETH as far as the law allows, open access under CC BY 4.0, contributor listing with opt-out, what students keep); confirmation is now section 4. Wording flagged for the ETH Legal Office.
- README: Section 9 Data (git for small files, Zenodo per course year for large files, GEO for sequencing); references to the sheet renamed; appendix item for the legal check, Zenodo record and download script.
- llms.txt, companion builder, Gantt workbook and builder follow the new name.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -1500,7 +1500,7 @@
       </c>
       <c r="B7" s="46" t="inlineStr">
         <is>
-          <t>Working in the lab and biosafety (Tea Kocijan), 10:30-12:00: Q&amp;A, then the safety sheet is signed</t>
+          <t>Working in the lab and biosafety (Tea Kocijan), 10:30-12:00: Q&amp;A, then the admission sheet (safety and data) is signed</t>
         </is>
       </c>
       <c r="C7" s="66" t="n"/>
@@ -1578,7 +1578,7 @@
       </c>
       <c r="B13" s="55" t="inlineStr">
         <is>
-          <t>Rooms, safety officer. Signed safety sheets collected at 12:00. Supervisors sit with their group from 14:00.</t>
+          <t>Rooms, safety officer. Signed admission sheets collected at 12:00. Supervisors sit with their group from 14:00.</t>
         </is>
       </c>
       <c r="C13" s="55" t="inlineStr">

</xml_diff>

<commit_message>
In silico arm as one standard scRNA-seq workflow: markers, M1/M2 scores, own signature
DESeq2 and the bulk dataset are gone. 03_markers.R finds the markers of the
macrophage clusters and asks students to name their M1 and M2 cluster before any
score. 04_m1_m2_score.R scores every cell with classic M1/M2 markers and with the
IFNγ and IL-4 consensus of Colombo et al. 2024 (supplementary table S1, top 30),
other cells as the control. 05_own_signature.R is a template for a signature from
the single-cell literature, for the poster. Setup: DESeq2/BiocManager out, readxl in.
Potential extensions in code/scrnaseq/README.md: take the workflow to an organ or
disease of your own choice, with CellChat, NicheNet and monocle3. Course script
Experiment 2, extension table, open items, background and schedule texts
(Gantt workbook and gantt_build.py) follow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/tools/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -1098,7 +1098,7 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Week 1: environment and templates. Exp 2, the in silico comparison, runs through weeks 2 to 4. Week 2: scRNA-seq part 1 (QC) in the afternoon dry-lab slots, FlowJo on the own data. Week 3: scRNA-seq part 2 (signatures from the bulk RAW 264.7 dataset) during the challenge and the ELISA incubations, own ELISA data on Friday. Week 4: scRNA-seq part 3 (scoring of the tissue macrophages), wrap up of code, figures and poster.</t>
+          <t>Week 1: environment and templates. Exp 2, the in silico comparison, runs through weeks 2 to 4. Week 2: scRNA-seq part 1 (QC) in the afternoon dry-lab slots, FlowJo on the own data. Week 3: scRNA-seq part 2 (markers of the macrophage clusters, M1/M2 scores) during the challenge and the ELISA incubations, own ELISA data on Friday. Week 4: scRNA-seq part 3 (your own signature, for the poster), wrap up of code, figures and poster.</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>Dry lab: scRNA-seq part 1, load the preprocessed object, QC figure. If the bench runs over, the dry lab moves home.</t>
+          <t>Dry lab: scRNA-seq part 1, download and load the data, QC figure. If the bench runs over, the dry lab moves home.</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
@@ -2089,7 +2089,7 @@
       <c r="B10" s="65" t="n"/>
       <c r="C10" s="54" t="inlineStr">
         <is>
-          <t>Dry lab during the challenge: scRNA-seq part 2, signatures from the bulk RAW 264.7 dataset. TNF groups: harvest at 15:00, supernatants and lysates to the freezer.</t>
+          <t>Dry lab during the challenge: scRNA-seq part 2, markers of the macrophage clusters and the M1/M2 scores. TNF groups: harvest at 15:00, supernatants and lysates to the freezer.</t>
         </is>
       </c>
       <c r="D10" s="66" t="n"/>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C9" s="51" t="inlineStr">
         <is>
-          <t>Wrap up: code, figures and poster; scRNA-seq part 3, score the tissue macrophages</t>
+          <t>Wrap up: code, figures and poster; scRNA-seq part 3, your own signature for the poster</t>
         </is>
       </c>
       <c r="D9" s="51" t="inlineStr">

</xml_diff>